<commit_message>
refactor(rating): 删除 tblevelrating 表与评级生成代码
2026-11-01 用户定规：星级评分体系整体下线，通关一律记固定星级。本笔只落地
「配置表 + Luban 生成代码」这一层，运行时与 UI 改动跟随后续提交。

- __tables__.xlsx 注销 tblevelrating，删除 30 张 Levels/Lxx/LevelRating.xlsx
- 删除 Assets/Gen 下 TBLevelRating.cs / LevelRating.cs 及 meta，Tables.cs 去掉该表
- Configs 移除 RatingTable、VerifyRatingContent、CalculateRuntimeContentHash、
  ValidateRatingPlan 调用链与 RatingContentVerified 标志
- ResTable 移除 tblevelrating 地址，Configs.EditorCandidates 的候选表清单同步

改表流程不再需要重封 runtimeContentHash，也不会再出现 content hash mismatch 拦关。
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/__tables__.xlsx
+++ b/Luban/Config/Datas/__tables__.xlsx
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="7"/>
   <cols>
     <col width="21.25" customWidth="1" style="2" min="1" max="1"/>
@@ -1425,50 +1425,25 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Level performance rating</t>
+          <t>每关玩法常数（2026-10-30 从 Global 拆出）</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>TBLevelRating</t>
+          <t>TBLevelRules</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t>LevelRating</t>
-        </is>
-      </c>
-      <c r="D14" s="0" t="b">
-        <v>1</v>
+          <t>LevelRules</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
-        <is>
-          <t>Levels/L01/LevelRating.xlsx,Levels/L02/LevelRating.xlsx,Levels/L03/LevelRating.xlsx,Levels/L04/LevelRating.xlsx,Levels/L05/LevelRating.xlsx,Levels/L06/LevelRating.xlsx,Levels/L07/LevelRating.xlsx,Levels/L08/LevelRating.xlsx,Levels/L09/LevelRating.xlsx,Levels/L10/LevelRating.xlsx,Levels/L11/LevelRating.xlsx,Levels/L12/LevelRating.xlsx,Levels/L13/LevelRating.xlsx,Levels/L14/LevelRating.xlsx,Levels/L15/LevelRating.xlsx,Levels/L16/LevelRating.xlsx,Levels/L17/LevelRating.xlsx,Levels/L18/LevelRating.xlsx,Levels/L19/LevelRating.xlsx,Levels/L20/LevelRating.xlsx,Levels/L21/LevelRating.xlsx,Levels/L22/LevelRating.xlsx,Levels/L23/LevelRating.xlsx,Levels/L24/LevelRating.xlsx,Levels/L25/LevelRating.xlsx,Levels/L26/LevelRating.xlsx,Levels/L27/LevelRating.xlsx,Levels/L28/LevelRating.xlsx,Levels/L29/LevelRating.xlsx,Levels/L30/LevelRating.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="0" t="inlineStr">
-        <is>
-          <t>每关玩法常数（2026-10-30 从 Global 拆出）</t>
-        </is>
-      </c>
-      <c r="B15" s="0" t="inlineStr">
-        <is>
-          <t>TBLevelRules</t>
-        </is>
-      </c>
-      <c r="C15" s="0" t="inlineStr">
-        <is>
-          <t>LevelRules</t>
-        </is>
-      </c>
-      <c r="D15" s="0" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>Levels/L01/LevelRules.xlsx,Levels/L02/LevelRules.xlsx,Levels/L03/LevelRules.xlsx,Levels/L04/LevelRules.xlsx,Levels/L05/LevelRules.xlsx,Levels/L06/LevelRules.xlsx,Levels/L07/LevelRules.xlsx,Levels/L08/LevelRules.xlsx,Levels/L09/LevelRules.xlsx,Levels/L10/LevelRules.xlsx,Levels/L11/LevelRules.xlsx,Levels/L12/LevelRules.xlsx,Levels/L13/LevelRules.xlsx,Levels/L14/LevelRules.xlsx,Levels/L15/LevelRules.xlsx,Levels/L16/LevelRules.xlsx,Levels/L17/LevelRules.xlsx,Levels/L18/LevelRules.xlsx,Levels/L19/LevelRules.xlsx,Levels/L20/LevelRules.xlsx,Levels/L21/LevelRules.xlsx,Levels/L22/LevelRules.xlsx,Levels/L23/LevelRules.xlsx,Levels/L24/LevelRules.xlsx,Levels/L25/LevelRules.xlsx,Levels/L26/LevelRules.xlsx,Levels/L27/LevelRules.xlsx,Levels/L28/LevelRules.xlsx,Levels/L29/LevelRules.xlsx,Levels/L30/LevelRules.xlsx</t>
         </is>

</xml_diff>